<commit_message>
improving reports pending selection
</commit_message>
<xml_diff>
--- a/data/CARGA - 2QZ JULHO 2026 - VEXPENSES - API.xlsx
+++ b/data/CARGA - 2QZ JULHO 2026 - VEXPENSES - API.xlsx
@@ -3745,10 +3745,10 @@
         </is>
       </c>
       <c r="I59" s="3" t="n">
-        <v>798.6</v>
+        <v>269.52</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>-798.6</v>
+        <v>-269.52</v>
       </c>
       <c r="K59" s="3" t="n">
         <v>0</v>
@@ -3867,10 +3867,10 @@
         </is>
       </c>
       <c r="I61" s="3" t="n">
-        <v>2364.12</v>
+        <v>965.45</v>
       </c>
       <c r="J61" s="3" t="n">
-        <v>-2364.12</v>
+        <v>-965.45</v>
       </c>
       <c r="K61" s="3" t="inlineStr"/>
       <c r="L61" s="3" t="n">
@@ -6771,10 +6771,10 @@
         </is>
       </c>
       <c r="I110" s="3" t="n">
-        <v>844.2</v>
+        <v>240.2</v>
       </c>
       <c r="J110" s="3" t="n">
-        <v>-844.2</v>
+        <v>-240.2</v>
       </c>
       <c r="K110" s="3" t="n">
         <v>700</v>
@@ -10176,7 +10176,7 @@
         <v>0</v>
       </c>
       <c r="J168" s="3" t="n">
-        <v>1306.57</v>
+        <v>943.97</v>
       </c>
       <c r="K168" s="3" t="n">
         <v>2000</v>
@@ -10186,13 +10186,13 @@
       </c>
       <c r="M168" s="3" t="inlineStr"/>
       <c r="N168" s="3" t="n">
-        <v>688.1799999999999</v>
+        <v>1050.78</v>
       </c>
       <c r="O168" s="3" t="n">
         <v>0</v>
       </c>
       <c r="P168" s="3" t="n">
-        <v>688.1799999999999</v>
+        <v>1050.78</v>
       </c>
       <c r="Q168" s="2" t="inlineStr">
         <is>
@@ -13435,10 +13435,10 @@
         </is>
       </c>
       <c r="I221" s="3" t="n">
-        <v>59.71</v>
+        <v>124.71</v>
       </c>
       <c r="J221" s="3" t="n">
-        <v>-59.71</v>
+        <v>-124.71</v>
       </c>
       <c r="K221" s="3" t="n">
         <v>675</v>
@@ -19603,10 +19603,10 @@
         </is>
       </c>
       <c r="I325" s="3" t="n">
-        <v>1056.93</v>
+        <v>2206.93</v>
       </c>
       <c r="J325" s="3" t="n">
-        <v>-1056.93</v>
+        <v>-2206.93</v>
       </c>
       <c r="K325" s="3" t="n">
         <v>500</v>
@@ -22210,7 +22210,7 @@
         <v>0</v>
       </c>
       <c r="J369" s="3" t="n">
-        <v>182</v>
+        <v>150.2</v>
       </c>
       <c r="K369" s="3" t="inlineStr"/>
       <c r="L369" s="3" t="n">
@@ -22218,7 +22218,7 @@
       </c>
       <c r="M369" s="3" t="inlineStr"/>
       <c r="N369" s="3" t="n">
-        <v>-182</v>
+        <v>-150.2</v>
       </c>
       <c r="O369" s="3" t="n">
         <v>0</v>
@@ -23081,10 +23081,10 @@
         </is>
       </c>
       <c r="I385" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="J385" s="3" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="K385" s="3" t="n">
         <v>800</v>
@@ -23094,13 +23094,13 @@
       </c>
       <c r="M385" s="3" t="inlineStr"/>
       <c r="N385" s="3" t="n">
-        <v>619.9400000000001</v>
+        <v>799.9400000000001</v>
       </c>
       <c r="O385" s="3" t="n">
         <v>0</v>
       </c>
       <c r="P385" s="3" t="n">
-        <v>619.9400000000001</v>
+        <v>799.9400000000001</v>
       </c>
       <c r="Q385" s="2" t="inlineStr">
         <is>
@@ -31362,7 +31362,7 @@
         <v>0</v>
       </c>
       <c r="J522" s="3" t="n">
-        <v>825.9</v>
+        <v>677.2</v>
       </c>
       <c r="K522" s="3" t="n">
         <v>1000</v>
@@ -31372,13 +31372,13 @@
       </c>
       <c r="M522" s="3" t="inlineStr"/>
       <c r="N522" s="3" t="n">
-        <v>173.8</v>
+        <v>322.5</v>
       </c>
       <c r="O522" s="3" t="n">
         <v>0</v>
       </c>
       <c r="P522" s="3" t="n">
-        <v>173.8</v>
+        <v>322.5</v>
       </c>
       <c r="Q522" s="2" t="inlineStr">
         <is>
@@ -36807,10 +36807,10 @@
         </is>
       </c>
       <c r="I613" s="3" t="n">
-        <v>95.65000000000001</v>
+        <v>-0</v>
       </c>
       <c r="J613" s="3" t="n">
-        <v>-95.65000000000001</v>
+        <v>0</v>
       </c>
       <c r="K613" s="3" t="inlineStr"/>
       <c r="L613" s="3" t="n">
@@ -37173,10 +37173,10 @@
         </is>
       </c>
       <c r="I619" s="3" t="n">
-        <v>12062.79</v>
+        <v>1679.09</v>
       </c>
       <c r="J619" s="3" t="n">
-        <v>-12062.79</v>
+        <v>-1679.09</v>
       </c>
       <c r="K619" s="3" t="inlineStr"/>
       <c r="L619" s="3" t="n">
@@ -38521,10 +38521,10 @@
         </is>
       </c>
       <c r="I642" s="3" t="n">
-        <v>280</v>
+        <v>953.8200000000001</v>
       </c>
       <c r="J642" s="3" t="n">
-        <v>-280</v>
+        <v>-953.8200000000001</v>
       </c>
       <c r="K642" s="3" t="n">
         <v>600</v>
@@ -40330,7 +40330,7 @@
         <v>0</v>
       </c>
       <c r="J672" s="3" t="n">
-        <v>241.63</v>
+        <v>171.63</v>
       </c>
       <c r="K672" s="3" t="n">
         <v>160</v>
@@ -40340,7 +40340,7 @@
       </c>
       <c r="M672" s="3" t="inlineStr"/>
       <c r="N672" s="3" t="n">
-        <v>-81.63</v>
+        <v>-11.63</v>
       </c>
       <c r="O672" s="3" t="n">
         <v>0</v>
@@ -42147,10 +42147,10 @@
         </is>
       </c>
       <c r="I702" s="3" t="n">
-        <v>1628.21</v>
+        <v>1833.21</v>
       </c>
       <c r="J702" s="3" t="n">
-        <v>-1628.21</v>
+        <v>-1833.21</v>
       </c>
       <c r="K702" s="3" t="n">
         <v>2000</v>
@@ -42572,7 +42572,7 @@
         <v>0</v>
       </c>
       <c r="J709" s="3" t="n">
-        <v>3914.46</v>
+        <v>3434.46</v>
       </c>
       <c r="K709" s="3" t="n">
         <v>4000</v>
@@ -42582,13 +42582,13 @@
       </c>
       <c r="M709" s="3" t="inlineStr"/>
       <c r="N709" s="3" t="n">
-        <v>-171.77</v>
+        <v>308.23</v>
       </c>
       <c r="O709" s="3" t="n">
         <v>0</v>
       </c>
       <c r="P709" s="3" t="n">
-        <v>0</v>
+        <v>308.23</v>
       </c>
       <c r="Q709" s="2" t="inlineStr">
         <is>
@@ -44369,10 +44369,10 @@
         </is>
       </c>
       <c r="I739" s="3" t="n">
-        <v>0</v>
+        <v>482.68</v>
       </c>
       <c r="J739" s="3" t="n">
-        <v>515.22</v>
+        <v>-482.68</v>
       </c>
       <c r="K739" s="3" t="n">
         <v>1500</v>
@@ -44382,13 +44382,13 @@
       </c>
       <c r="M739" s="3" t="inlineStr"/>
       <c r="N739" s="3" t="n">
-        <v>948.78</v>
+        <v>1464</v>
       </c>
       <c r="O739" s="3" t="n">
         <v>0</v>
       </c>
       <c r="P739" s="3" t="n">
-        <v>948.78</v>
+        <v>1464</v>
       </c>
       <c r="Q739" s="2" t="inlineStr">
         <is>
@@ -44620,7 +44620,7 @@
         <v>0</v>
       </c>
       <c r="J743" s="3" t="n">
-        <v>2168.86</v>
+        <v>1932.06</v>
       </c>
       <c r="K743" s="3" t="n">
         <v>0</v>
@@ -44630,7 +44630,7 @@
       </c>
       <c r="M743" s="3" t="inlineStr"/>
       <c r="N743" s="3" t="n">
-        <v>-2169.74</v>
+        <v>-1932.94</v>
       </c>
       <c r="O743" s="3" t="n">
         <v>0</v>

</xml_diff>